<commit_message>
Add ri_treatment_area to samplingFeatureTypes.xml; retire rigid_inclusion_system; fix stale targetSFType xpath
RigidInclusionSystem is now an AbstractSamplingFeatureGroup, not a sampling feature (S10r),
so rigid_inclusion_system no longer belongs in this dictionary. RITreatedArea substitutes
AbstractPlanarSamplingFeature directly and had no code of its own - added as ri_treatment_area.

Also repoints every entry's sourceElementXpath from the retired TargetSamplingFeatureType/
targetSFType to the real consumer, AbstractSamplingFeatureDesignType/samplingFeatureType, and
renames the dictionary's own root gml:id to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/samplingFeatureTypes.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/samplingFeatureTypes.xlsx
@@ -970,7 +970,7 @@
     <row r="3" ht="154" customFormat="1" customHeight="1" s="2">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>targetSFType</t>
+          <t>samplingFeatureType</t>
         </is>
       </c>
       <c r="C3" s="12" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes naming the kind of sampling feature planned. These codes are used for the value of the targetSFType property of diggs:TargetSamplingFeature and its specializations (diggs:TargetBorehole, diggs:TargetInstallation). Covers both plain sampling features and installation-type sampling features in one vocabulary, since an installation is itself a sampling feature in DIGGS (diggs:AbstractLinearInstallation and diggs:AbstractPlanarInstallation both substitute diggs:AbstractSamplingFeature directly) - there is no separate installation-type head to key a second dictionary on. The list is every concrete sampling feature kind in the schema as of 3.1-dev; a future schema addition that substitutes diggs:AbstractSamplingFeature should get a matching entry here.</t>
+          <t>Codes naming the kind of sampling feature a design applies to. Used for the value of samplingFeatureType on AbstractSamplingFeatureDesignType and its specializations. Covers both plain sampling features and installation-type sampling features in one vocabulary, since an installation is itself a sampling feature in DIGGS (AbstractLinearInstallation and AbstractPlanarInstallation both substitute AbstractSamplingFeature directly) - there is no separate installation-type head to key a second dictionary on. The list is every concrete sampling feature kind in the schema; a future schema addition that substitutes AbstractSamplingFeature should get a matching entry here.</t>
         </is>
       </c>
     </row>
@@ -1572,17 +1572,17 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>rigid_inclusion_system</t>
+          <t>ri_treatment_area</t>
         </is>
       </c>
       <c r="C20" s="18" t="inlineStr">
         <is>
-          <t>Rigid inclusion system</t>
+          <t>RI treatment area</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>A top-level, complex sampling feature describing the components of a rigid inclusion system - the load transfer platform and the individual rigid inclusion columns constructed within the soil below it.</t>
+          <t>The area of a site treated by a rigid inclusion ground improvement program - the ground improvement footprint that includes the rigid inclusion columns and may extend beyond any associated foundation or embankment.</t>
         </is>
       </c>
       <c r="E20" s="18" t="inlineStr">
@@ -1860,7 +1860,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2143,12 +2143,12 @@
       </c>
       <c r="B20" s="20" t="inlineStr">
         <is>
-          <t>rigid_inclusion_system</t>
+          <t>ri_treatment_area</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>//diggs:targetSFType</t>
+          <t>//diggs:samplingFeatureType</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
samplingFeatureTypes: bind to appliesToFeatureType on program specifications (second Occurrence per entry, 20 entries)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/samplingFeatureTypes.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/samplingFeatureTypes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes naming the kind of sampling feature a design applies to. Used for the value of samplingFeatureType on AbstractSamplingFeatureDesignType and its specializations. Covers both plain sampling features and installation-type sampling features in one vocabulary, since an installation is itself a sampling feature in DIGGS (AbstractLinearInstallation and AbstractPlanarInstallation both substitute AbstractSamplingFeature directly) - there is no separate installation-type head to key a second dictionary on. The list is every concrete sampling feature kind in the schema; a future schema addition that substitutes AbstractSamplingFeature should get a matching entry here.</t>
+          <t>Codes naming the kind of sampling feature a design applies to. Used for the value of samplingFeatureType on AbstractSamplingFeatureDesignType and its specializations, and of appliesToFeatureType on AbstractProgramSpecificationType and its specializations. Covers both plain sampling features and installation-type sampling features in one vocabulary, since an installation is itself a sampling feature in DIGGS (AbstractLinearInstallation and AbstractPlanarInstallation both substitute AbstractSamplingFeature directly) - there is no separate installation-type head to key a second dictionary on. The list is every concrete sampling feature kind in the schema; a future schema addition that substitutes AbstractSamplingFeature should get a matching entry here.</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="6.83203125" customWidth="1" min="1" max="1"/>
@@ -2173,112 +2173,320 @@
         <f>IF(ISNA(VLOOKUP(B22,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B22" s="20" t="n"/>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>borehole</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
         <f>IF(ISNA(VLOOKUP(B23,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B23" s="20" t="n"/>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>sounding</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
         <f>IF(ISNA(VLOOKUP(B24,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B24" s="2" t="n"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>trial_pit</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
         <f>IF(ISNA(VLOOKUP(B25,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B25" s="2" t="n"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>transect</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
         <f>IF(ISNA(VLOOKUP(B26,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B26" s="2" t="n"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>gp_trackline</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
         <f>IF(ISNA(VLOOKUP(B27,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B27" s="13" t="n"/>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>grout_trench_cutoff_wall</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
         <f>IF(ISNA(VLOOKUP(B28,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B28" s="13" t="n"/>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>well</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
         <f>IF(ISNA(VLOOKUP(B29,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B29" s="13" t="n"/>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>steel_h_pile</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
         <f>IF(ISNA(VLOOKUP(B30,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B30" s="13" t="n"/>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>steel_pipe_pile</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
         <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B31" s="13" t="n"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>concrete_pile</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
         <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B32" s="13" t="n"/>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>timber_pile</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
         <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>gp_multi_track</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
         <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>station</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
         <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B35" s="13" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>ri_column</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
         <f>IF(ISNA(VLOOKUP(B36,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B36" s="13" t="n"/>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>gp_areal_survey</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
         <f>IF(ISNA(VLOOKUP(B37,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B37" s="2" t="n"/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>planar_sampling_feature</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <f>IF(ISNA(VLOOKUP(B38,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>trench_wall</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <f>IF(ISNA(VLOOKUP(B39,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>load_transfer_platform</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <f>IF(ISNA(VLOOKUP(B40,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>ri_treatment_area</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <f>IF(ISNA(VLOOKUP(B41,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>volumetric_sampling_feature</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>//diggs:appliesToFeatureType</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>